<commit_message>
Add calendar events for DG_GEN, QJB, STM, MCU, DBF, DRM, NFS in September 2026
</commit_message>
<xml_diff>
--- a/RPM_Dashboard_InputData_v10.xlsx
+++ b/RPM_Dashboard_InputData_v10.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/841abc774317df50/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{39D72C63-0BE4-4977-B56D-A0E79FB87673}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="11_F7FC1742F3B5B5C4C1F9F036D5AEF24CB7B4329D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D908A63-2023-4E08-974D-B565C1E909B5}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GUIDE" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1786" uniqueCount="1028">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1835" uniqueCount="1037">
   <si>
     <t>RADAR PREVENTIVE MAINTENANCE DASHBOARD</t>
   </si>
@@ -3126,13 +3126,43 @@
     <t xml:space="preserve">Display Console </t>
   </si>
   <si>
-    <t xml:space="preserve">tested it </t>
+    <t>task_Description</t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>DG Gen – Annual</t>
+  </si>
+  <si>
+    <t>Tuesday</t>
+  </si>
+  <si>
+    <t>QJB – Quarterly</t>
+  </si>
+  <si>
+    <t>STM – Quarterly</t>
+  </si>
+  <si>
+    <t>MCU – Annual</t>
+  </si>
+  <si>
+    <t>DBF – Quarterly</t>
+  </si>
+  <si>
+    <t>DRM – Quarterly</t>
+  </si>
+  <si>
+    <t>NFS – Quarterly</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="169" formatCode="[$-14009]yyyy/mm/dd;@"/>
+  </numFmts>
   <fonts count="34" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -3512,7 +3542,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -3563,11 +3593,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFAABBCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFAABBCC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -3829,32 +3870,23 @@
     <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3868,6 +3900,15 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3877,6 +3918,10 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3960,6 +4005,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4172,72 +4221,72 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
-      <c r="B2" s="106" t="s">
+      <c r="B2" s="103" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="106"/>
-      <c r="D2" s="106"/>
-      <c r="E2" s="106"/>
-      <c r="F2" s="106"/>
-      <c r="G2" s="106"/>
-      <c r="H2" s="106"/>
-      <c r="I2" s="106"/>
-      <c r="J2" s="106"/>
-      <c r="K2" s="106"/>
-      <c r="L2" s="106"/>
-      <c r="M2" s="106"/>
+      <c r="C2" s="103"/>
+      <c r="D2" s="103"/>
+      <c r="E2" s="103"/>
+      <c r="F2" s="103"/>
+      <c r="G2" s="103"/>
+      <c r="H2" s="103"/>
+      <c r="I2" s="103"/>
+      <c r="J2" s="103"/>
+      <c r="K2" s="103"/>
+      <c r="L2" s="103"/>
+      <c r="M2" s="103"/>
       <c r="N2" s="1"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
-      <c r="B3" s="106"/>
-      <c r="C3" s="106"/>
-      <c r="D3" s="106"/>
-      <c r="E3" s="106"/>
-      <c r="F3" s="106"/>
-      <c r="G3" s="106"/>
-      <c r="H3" s="106"/>
-      <c r="I3" s="106"/>
-      <c r="J3" s="106"/>
-      <c r="K3" s="106"/>
-      <c r="L3" s="106"/>
-      <c r="M3" s="106"/>
+      <c r="B3" s="103"/>
+      <c r="C3" s="103"/>
+      <c r="D3" s="103"/>
+      <c r="E3" s="103"/>
+      <c r="F3" s="103"/>
+      <c r="G3" s="103"/>
+      <c r="H3" s="103"/>
+      <c r="I3" s="103"/>
+      <c r="J3" s="103"/>
+      <c r="K3" s="103"/>
+      <c r="L3" s="103"/>
+      <c r="M3" s="103"/>
       <c r="N3" s="1"/>
     </row>
     <row r="4" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
-      <c r="B4" s="107" t="s">
+      <c r="B4" s="104" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="107"/>
-      <c r="D4" s="107"/>
-      <c r="E4" s="107"/>
-      <c r="F4" s="107"/>
-      <c r="G4" s="107"/>
-      <c r="H4" s="107"/>
-      <c r="I4" s="107"/>
-      <c r="J4" s="107"/>
-      <c r="K4" s="107"/>
-      <c r="L4" s="107"/>
-      <c r="M4" s="107"/>
+      <c r="C4" s="104"/>
+      <c r="D4" s="104"/>
+      <c r="E4" s="104"/>
+      <c r="F4" s="104"/>
+      <c r="G4" s="104"/>
+      <c r="H4" s="104"/>
+      <c r="I4" s="104"/>
+      <c r="J4" s="104"/>
+      <c r="K4" s="104"/>
+      <c r="L4" s="104"/>
+      <c r="M4" s="104"/>
       <c r="N4" s="1"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
-      <c r="B5" s="108" t="s">
+      <c r="B5" s="105" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="108"/>
-      <c r="D5" s="108"/>
-      <c r="E5" s="108"/>
-      <c r="F5" s="108"/>
-      <c r="G5" s="108"/>
-      <c r="H5" s="108"/>
-      <c r="I5" s="108"/>
-      <c r="J5" s="108"/>
-      <c r="K5" s="108"/>
-      <c r="L5" s="108"/>
-      <c r="M5" s="108"/>
+      <c r="C5" s="105"/>
+      <c r="D5" s="105"/>
+      <c r="E5" s="105"/>
+      <c r="F5" s="105"/>
+      <c r="G5" s="105"/>
+      <c r="H5" s="105"/>
+      <c r="I5" s="105"/>
+      <c r="J5" s="105"/>
+      <c r="K5" s="105"/>
+      <c r="L5" s="105"/>
+      <c r="M5" s="105"/>
       <c r="N5" s="1"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
@@ -4274,20 +4323,20 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
-      <c r="B8" s="109" t="s">
+      <c r="B8" s="106" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="109"/>
-      <c r="D8" s="109"/>
-      <c r="E8" s="109"/>
-      <c r="F8" s="109"/>
-      <c r="G8" s="109"/>
-      <c r="H8" s="109"/>
-      <c r="I8" s="109"/>
-      <c r="J8" s="109"/>
-      <c r="K8" s="109"/>
-      <c r="L8" s="109"/>
-      <c r="M8" s="109"/>
+      <c r="C8" s="106"/>
+      <c r="D8" s="106"/>
+      <c r="E8" s="106"/>
+      <c r="F8" s="106"/>
+      <c r="G8" s="106"/>
+      <c r="H8" s="106"/>
+      <c r="I8" s="106"/>
+      <c r="J8" s="106"/>
+      <c r="K8" s="106"/>
+      <c r="L8" s="106"/>
+      <c r="M8" s="106"/>
       <c r="N8" s="1"/>
     </row>
     <row r="9" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -4295,19 +4344,19 @@
       <c r="B9" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="105" t="s">
+      <c r="C9" s="107" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="105"/>
-      <c r="E9" s="105"/>
-      <c r="F9" s="105"/>
-      <c r="G9" s="105"/>
-      <c r="H9" s="105"/>
-      <c r="I9" s="105"/>
-      <c r="J9" s="105"/>
-      <c r="K9" s="105"/>
-      <c r="L9" s="105"/>
-      <c r="M9" s="105"/>
+      <c r="D9" s="107"/>
+      <c r="E9" s="107"/>
+      <c r="F9" s="107"/>
+      <c r="G9" s="107"/>
+      <c r="H9" s="107"/>
+      <c r="I9" s="107"/>
+      <c r="J9" s="107"/>
+      <c r="K9" s="107"/>
+      <c r="L9" s="107"/>
+      <c r="M9" s="107"/>
       <c r="N9" s="1"/>
     </row>
     <row r="10" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -4315,19 +4364,19 @@
       <c r="B10" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="105" t="s">
+      <c r="C10" s="107" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="105"/>
-      <c r="E10" s="105"/>
-      <c r="F10" s="105"/>
-      <c r="G10" s="105"/>
-      <c r="H10" s="105"/>
-      <c r="I10" s="105"/>
-      <c r="J10" s="105"/>
-      <c r="K10" s="105"/>
-      <c r="L10" s="105"/>
-      <c r="M10" s="105"/>
+      <c r="D10" s="107"/>
+      <c r="E10" s="107"/>
+      <c r="F10" s="107"/>
+      <c r="G10" s="107"/>
+      <c r="H10" s="107"/>
+      <c r="I10" s="107"/>
+      <c r="J10" s="107"/>
+      <c r="K10" s="107"/>
+      <c r="L10" s="107"/>
+      <c r="M10" s="107"/>
       <c r="N10" s="1"/>
     </row>
     <row r="11" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -4335,19 +4384,19 @@
       <c r="B11" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="105" t="s">
+      <c r="C11" s="107" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="105"/>
-      <c r="E11" s="105"/>
-      <c r="F11" s="105"/>
-      <c r="G11" s="105"/>
-      <c r="H11" s="105"/>
-      <c r="I11" s="105"/>
-      <c r="J11" s="105"/>
-      <c r="K11" s="105"/>
-      <c r="L11" s="105"/>
-      <c r="M11" s="105"/>
+      <c r="D11" s="107"/>
+      <c r="E11" s="107"/>
+      <c r="F11" s="107"/>
+      <c r="G11" s="107"/>
+      <c r="H11" s="107"/>
+      <c r="I11" s="107"/>
+      <c r="J11" s="107"/>
+      <c r="K11" s="107"/>
+      <c r="L11" s="107"/>
+      <c r="M11" s="107"/>
       <c r="N11" s="1"/>
     </row>
     <row r="12" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -4355,19 +4404,19 @@
       <c r="B12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="105" t="s">
+      <c r="C12" s="107" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="105"/>
-      <c r="E12" s="105"/>
-      <c r="F12" s="105"/>
-      <c r="G12" s="105"/>
-      <c r="H12" s="105"/>
-      <c r="I12" s="105"/>
-      <c r="J12" s="105"/>
-      <c r="K12" s="105"/>
-      <c r="L12" s="105"/>
-      <c r="M12" s="105"/>
+      <c r="D12" s="107"/>
+      <c r="E12" s="107"/>
+      <c r="F12" s="107"/>
+      <c r="G12" s="107"/>
+      <c r="H12" s="107"/>
+      <c r="I12" s="107"/>
+      <c r="J12" s="107"/>
+      <c r="K12" s="107"/>
+      <c r="L12" s="107"/>
+      <c r="M12" s="107"/>
       <c r="N12" s="1"/>
     </row>
     <row r="13" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -4375,19 +4424,19 @@
       <c r="B13" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="105" t="s">
+      <c r="C13" s="107" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="105"/>
-      <c r="E13" s="105"/>
-      <c r="F13" s="105"/>
-      <c r="G13" s="105"/>
-      <c r="H13" s="105"/>
-      <c r="I13" s="105"/>
-      <c r="J13" s="105"/>
-      <c r="K13" s="105"/>
-      <c r="L13" s="105"/>
-      <c r="M13" s="105"/>
+      <c r="D13" s="107"/>
+      <c r="E13" s="107"/>
+      <c r="F13" s="107"/>
+      <c r="G13" s="107"/>
+      <c r="H13" s="107"/>
+      <c r="I13" s="107"/>
+      <c r="J13" s="107"/>
+      <c r="K13" s="107"/>
+      <c r="L13" s="107"/>
+      <c r="M13" s="107"/>
       <c r="N13" s="1"/>
     </row>
     <row r="14" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -4395,19 +4444,19 @@
       <c r="B14" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="105" t="s">
+      <c r="C14" s="107" t="s">
         <v>15</v>
       </c>
-      <c r="D14" s="105"/>
-      <c r="E14" s="105"/>
-      <c r="F14" s="105"/>
-      <c r="G14" s="105"/>
-      <c r="H14" s="105"/>
-      <c r="I14" s="105"/>
-      <c r="J14" s="105"/>
-      <c r="K14" s="105"/>
-      <c r="L14" s="105"/>
-      <c r="M14" s="105"/>
+      <c r="D14" s="107"/>
+      <c r="E14" s="107"/>
+      <c r="F14" s="107"/>
+      <c r="G14" s="107"/>
+      <c r="H14" s="107"/>
+      <c r="I14" s="107"/>
+      <c r="J14" s="107"/>
+      <c r="K14" s="107"/>
+      <c r="L14" s="107"/>
+      <c r="M14" s="107"/>
       <c r="N14" s="1"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
@@ -4428,20 +4477,20 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="104" t="s">
+      <c r="B16" s="108" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="104"/>
-      <c r="D16" s="104"/>
-      <c r="E16" s="104"/>
-      <c r="F16" s="104"/>
-      <c r="G16" s="104"/>
-      <c r="H16" s="104"/>
-      <c r="I16" s="104"/>
-      <c r="J16" s="104"/>
-      <c r="K16" s="104"/>
-      <c r="L16" s="104"/>
-      <c r="M16" s="104"/>
+      <c r="C16" s="108"/>
+      <c r="D16" s="108"/>
+      <c r="E16" s="108"/>
+      <c r="F16" s="108"/>
+      <c r="G16" s="108"/>
+      <c r="H16" s="108"/>
+      <c r="I16" s="108"/>
+      <c r="J16" s="108"/>
+      <c r="K16" s="108"/>
+      <c r="L16" s="108"/>
+      <c r="M16" s="108"/>
       <c r="N16" s="1"/>
     </row>
     <row r="17" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4682,20 +4731,20 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
-      <c r="B28" s="104" t="s">
+      <c r="B28" s="108" t="s">
         <v>47</v>
       </c>
-      <c r="C28" s="104"/>
-      <c r="D28" s="104"/>
-      <c r="E28" s="104"/>
-      <c r="F28" s="104"/>
-      <c r="G28" s="104"/>
-      <c r="H28" s="104"/>
-      <c r="I28" s="104"/>
-      <c r="J28" s="104"/>
-      <c r="K28" s="104"/>
-      <c r="L28" s="104"/>
-      <c r="M28" s="104"/>
+      <c r="C28" s="108"/>
+      <c r="D28" s="108"/>
+      <c r="E28" s="108"/>
+      <c r="F28" s="108"/>
+      <c r="G28" s="108"/>
+      <c r="H28" s="108"/>
+      <c r="I28" s="108"/>
+      <c r="J28" s="108"/>
+      <c r="K28" s="108"/>
+      <c r="L28" s="108"/>
+      <c r="M28" s="108"/>
       <c r="N28" s="1"/>
     </row>
     <row r="29" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4706,18 +4755,18 @@
       <c r="C29" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="D29" s="103" t="s">
+      <c r="D29" s="109" t="s">
         <v>50</v>
       </c>
-      <c r="E29" s="103"/>
-      <c r="F29" s="103"/>
-      <c r="G29" s="103"/>
-      <c r="H29" s="103"/>
-      <c r="I29" s="103"/>
-      <c r="J29" s="103"/>
-      <c r="K29" s="103"/>
-      <c r="L29" s="103"/>
-      <c r="M29" s="103"/>
+      <c r="E29" s="109"/>
+      <c r="F29" s="109"/>
+      <c r="G29" s="109"/>
+      <c r="H29" s="109"/>
+      <c r="I29" s="109"/>
+      <c r="J29" s="109"/>
+      <c r="K29" s="109"/>
+      <c r="L29" s="109"/>
+      <c r="M29" s="109"/>
       <c r="N29" s="1"/>
     </row>
     <row r="30" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4728,18 +4777,18 @@
       <c r="C30" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="D30" s="103" t="s">
+      <c r="D30" s="109" t="s">
         <v>52</v>
       </c>
-      <c r="E30" s="103"/>
-      <c r="F30" s="103"/>
-      <c r="G30" s="103"/>
-      <c r="H30" s="103"/>
-      <c r="I30" s="103"/>
-      <c r="J30" s="103"/>
-      <c r="K30" s="103"/>
-      <c r="L30" s="103"/>
-      <c r="M30" s="103"/>
+      <c r="E30" s="109"/>
+      <c r="F30" s="109"/>
+      <c r="G30" s="109"/>
+      <c r="H30" s="109"/>
+      <c r="I30" s="109"/>
+      <c r="J30" s="109"/>
+      <c r="K30" s="109"/>
+      <c r="L30" s="109"/>
+      <c r="M30" s="109"/>
       <c r="N30" s="1"/>
     </row>
     <row r="31" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4750,18 +4799,18 @@
       <c r="C31" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="D31" s="103" t="s">
+      <c r="D31" s="109" t="s">
         <v>54</v>
       </c>
-      <c r="E31" s="103"/>
-      <c r="F31" s="103"/>
-      <c r="G31" s="103"/>
-      <c r="H31" s="103"/>
-      <c r="I31" s="103"/>
-      <c r="J31" s="103"/>
-      <c r="K31" s="103"/>
-      <c r="L31" s="103"/>
-      <c r="M31" s="103"/>
+      <c r="E31" s="109"/>
+      <c r="F31" s="109"/>
+      <c r="G31" s="109"/>
+      <c r="H31" s="109"/>
+      <c r="I31" s="109"/>
+      <c r="J31" s="109"/>
+      <c r="K31" s="109"/>
+      <c r="L31" s="109"/>
+      <c r="M31" s="109"/>
       <c r="N31" s="1"/>
     </row>
     <row r="32" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4772,18 +4821,18 @@
       <c r="C32" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="D32" s="103" t="s">
+      <c r="D32" s="109" t="s">
         <v>56</v>
       </c>
-      <c r="E32" s="103"/>
-      <c r="F32" s="103"/>
-      <c r="G32" s="103"/>
-      <c r="H32" s="103"/>
-      <c r="I32" s="103"/>
-      <c r="J32" s="103"/>
-      <c r="K32" s="103"/>
-      <c r="L32" s="103"/>
-      <c r="M32" s="103"/>
+      <c r="E32" s="109"/>
+      <c r="F32" s="109"/>
+      <c r="G32" s="109"/>
+      <c r="H32" s="109"/>
+      <c r="I32" s="109"/>
+      <c r="J32" s="109"/>
+      <c r="K32" s="109"/>
+      <c r="L32" s="109"/>
+      <c r="M32" s="109"/>
       <c r="N32" s="1"/>
     </row>
     <row r="33" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4794,18 +4843,18 @@
       <c r="C33" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="D33" s="103" t="s">
+      <c r="D33" s="109" t="s">
         <v>58</v>
       </c>
-      <c r="E33" s="103"/>
-      <c r="F33" s="103"/>
-      <c r="G33" s="103"/>
-      <c r="H33" s="103"/>
-      <c r="I33" s="103"/>
-      <c r="J33" s="103"/>
-      <c r="K33" s="103"/>
-      <c r="L33" s="103"/>
-      <c r="M33" s="103"/>
+      <c r="E33" s="109"/>
+      <c r="F33" s="109"/>
+      <c r="G33" s="109"/>
+      <c r="H33" s="109"/>
+      <c r="I33" s="109"/>
+      <c r="J33" s="109"/>
+      <c r="K33" s="109"/>
+      <c r="L33" s="109"/>
+      <c r="M33" s="109"/>
       <c r="N33" s="1"/>
     </row>
     <row r="34" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4816,18 +4865,18 @@
       <c r="C34" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="D34" s="103" t="s">
+      <c r="D34" s="109" t="s">
         <v>60</v>
       </c>
-      <c r="E34" s="103"/>
-      <c r="F34" s="103"/>
-      <c r="G34" s="103"/>
-      <c r="H34" s="103"/>
-      <c r="I34" s="103"/>
-      <c r="J34" s="103"/>
-      <c r="K34" s="103"/>
-      <c r="L34" s="103"/>
-      <c r="M34" s="103"/>
+      <c r="E34" s="109"/>
+      <c r="F34" s="109"/>
+      <c r="G34" s="109"/>
+      <c r="H34" s="109"/>
+      <c r="I34" s="109"/>
+      <c r="J34" s="109"/>
+      <c r="K34" s="109"/>
+      <c r="L34" s="109"/>
+      <c r="M34" s="109"/>
       <c r="N34" s="1"/>
     </row>
     <row r="35" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4838,18 +4887,18 @@
       <c r="C35" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="D35" s="103" t="s">
+      <c r="D35" s="109" t="s">
         <v>62</v>
       </c>
-      <c r="E35" s="103"/>
-      <c r="F35" s="103"/>
-      <c r="G35" s="103"/>
-      <c r="H35" s="103"/>
-      <c r="I35" s="103"/>
-      <c r="J35" s="103"/>
-      <c r="K35" s="103"/>
-      <c r="L35" s="103"/>
-      <c r="M35" s="103"/>
+      <c r="E35" s="109"/>
+      <c r="F35" s="109"/>
+      <c r="G35" s="109"/>
+      <c r="H35" s="109"/>
+      <c r="I35" s="109"/>
+      <c r="J35" s="109"/>
+      <c r="K35" s="109"/>
+      <c r="L35" s="109"/>
+      <c r="M35" s="109"/>
       <c r="N35" s="1"/>
     </row>
     <row r="36" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4860,18 +4909,18 @@
       <c r="C36" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="D36" s="103" t="s">
+      <c r="D36" s="109" t="s">
         <v>64</v>
       </c>
-      <c r="E36" s="103"/>
-      <c r="F36" s="103"/>
-      <c r="G36" s="103"/>
-      <c r="H36" s="103"/>
-      <c r="I36" s="103"/>
-      <c r="J36" s="103"/>
-      <c r="K36" s="103"/>
-      <c r="L36" s="103"/>
-      <c r="M36" s="103"/>
+      <c r="E36" s="109"/>
+      <c r="F36" s="109"/>
+      <c r="G36" s="109"/>
+      <c r="H36" s="109"/>
+      <c r="I36" s="109"/>
+      <c r="J36" s="109"/>
+      <c r="K36" s="109"/>
+      <c r="L36" s="109"/>
+      <c r="M36" s="109"/>
       <c r="N36" s="1"/>
     </row>
     <row r="37" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4882,18 +4931,18 @@
       <c r="C37" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="D37" s="103" t="s">
+      <c r="D37" s="109" t="s">
         <v>66</v>
       </c>
-      <c r="E37" s="103"/>
-      <c r="F37" s="103"/>
-      <c r="G37" s="103"/>
-      <c r="H37" s="103"/>
-      <c r="I37" s="103"/>
-      <c r="J37" s="103"/>
-      <c r="K37" s="103"/>
-      <c r="L37" s="103"/>
-      <c r="M37" s="103"/>
+      <c r="E37" s="109"/>
+      <c r="F37" s="109"/>
+      <c r="G37" s="109"/>
+      <c r="H37" s="109"/>
+      <c r="I37" s="109"/>
+      <c r="J37" s="109"/>
+      <c r="K37" s="109"/>
+      <c r="L37" s="109"/>
+      <c r="M37" s="109"/>
       <c r="N37" s="1"/>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
@@ -5266,27 +5315,27 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="B2:M3"/>
-    <mergeCell ref="B4:M4"/>
-    <mergeCell ref="B5:M5"/>
-    <mergeCell ref="B8:M8"/>
-    <mergeCell ref="C9:M9"/>
-    <mergeCell ref="C10:M10"/>
-    <mergeCell ref="C11:M11"/>
-    <mergeCell ref="C12:M12"/>
-    <mergeCell ref="C13:M13"/>
-    <mergeCell ref="C14:M14"/>
-    <mergeCell ref="B16:M16"/>
-    <mergeCell ref="B28:M28"/>
-    <mergeCell ref="D29:M29"/>
-    <mergeCell ref="D30:M30"/>
-    <mergeCell ref="D31:M31"/>
     <mergeCell ref="D37:M37"/>
     <mergeCell ref="D32:M32"/>
     <mergeCell ref="D33:M33"/>
     <mergeCell ref="D34:M34"/>
     <mergeCell ref="D35:M35"/>
     <mergeCell ref="D36:M36"/>
+    <mergeCell ref="B16:M16"/>
+    <mergeCell ref="B28:M28"/>
+    <mergeCell ref="D29:M29"/>
+    <mergeCell ref="D30:M30"/>
+    <mergeCell ref="D31:M31"/>
+    <mergeCell ref="C10:M10"/>
+    <mergeCell ref="C11:M11"/>
+    <mergeCell ref="C12:M12"/>
+    <mergeCell ref="C13:M13"/>
+    <mergeCell ref="C14:M14"/>
+    <mergeCell ref="B2:M3"/>
+    <mergeCell ref="B4:M4"/>
+    <mergeCell ref="B5:M5"/>
+    <mergeCell ref="B8:M8"/>
+    <mergeCell ref="C9:M9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -5312,38 +5361,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="97" t="s">
         <v>975</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="101"/>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="101"/>
-      <c r="B2" s="101"/>
-      <c r="C2" s="101"/>
-      <c r="D2" s="101"/>
-      <c r="E2" s="101"/>
-      <c r="F2" s="101"/>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
+      <c r="A2" s="97"/>
+      <c r="B2" s="97"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="97"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="97"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="102" t="s">
+      <c r="A3" s="98" t="s">
         <v>976</v>
       </c>
-      <c r="B3" s="102"/>
-      <c r="C3" s="102"/>
-      <c r="D3" s="102"/>
-      <c r="E3" s="102"/>
-      <c r="F3" s="102"/>
-      <c r="G3" s="102"/>
-      <c r="H3" s="102"/>
+      <c r="B3" s="98"/>
+      <c r="C3" s="98"/>
+      <c r="D3" s="98"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="98"/>
     </row>
     <row r="4" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">
@@ -5614,56 +5663,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="97" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="101"/>
-      <c r="I1" s="101"/>
-      <c r="J1" s="101"/>
-      <c r="K1" s="101"/>
-      <c r="L1" s="101"/>
-      <c r="M1" s="101"/>
-      <c r="N1" s="101"/>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
     </row>
     <row r="2" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="101"/>
-      <c r="B2" s="101"/>
-      <c r="C2" s="101"/>
-      <c r="D2" s="101"/>
-      <c r="E2" s="101"/>
-      <c r="F2" s="101"/>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="101"/>
-      <c r="J2" s="101"/>
-      <c r="K2" s="101"/>
-      <c r="L2" s="101"/>
-      <c r="M2" s="101"/>
-      <c r="N2" s="101"/>
+      <c r="A2" s="97"/>
+      <c r="B2" s="97"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="97"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="97"/>
+      <c r="I2" s="97"/>
+      <c r="J2" s="97"/>
+      <c r="K2" s="97"/>
+      <c r="L2" s="97"/>
+      <c r="M2" s="97"/>
+      <c r="N2" s="97"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="102" t="s">
+      <c r="A3" s="98" t="s">
         <v>68</v>
       </c>
-      <c r="B3" s="102"/>
-      <c r="C3" s="102"/>
-      <c r="D3" s="102"/>
-      <c r="E3" s="102"/>
-      <c r="F3" s="102"/>
-      <c r="G3" s="102"/>
-      <c r="H3" s="102"/>
-      <c r="I3" s="102"/>
-      <c r="J3" s="102"/>
-      <c r="K3" s="102"/>
-      <c r="L3" s="102"/>
-      <c r="M3" s="102"/>
-      <c r="N3" s="102"/>
+      <c r="B3" s="98"/>
+      <c r="C3" s="98"/>
+      <c r="D3" s="98"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="98"/>
+      <c r="I3" s="98"/>
+      <c r="J3" s="98"/>
+      <c r="K3" s="98"/>
+      <c r="L3" s="98"/>
+      <c r="M3" s="98"/>
+      <c r="N3" s="98"/>
     </row>
     <row r="4" spans="1:14" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">
@@ -6297,62 +6346,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="97" t="s">
         <v>140</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="101"/>
-      <c r="I1" s="101"/>
-      <c r="J1" s="101"/>
-      <c r="K1" s="101"/>
-      <c r="L1" s="101"/>
-      <c r="M1" s="101"/>
-      <c r="N1" s="101"/>
-      <c r="O1" s="101"/>
-      <c r="P1" s="101"/>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A2" s="101"/>
-      <c r="B2" s="101"/>
-      <c r="C2" s="101"/>
-      <c r="D2" s="101"/>
-      <c r="E2" s="101"/>
-      <c r="F2" s="101"/>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="101"/>
-      <c r="J2" s="101"/>
-      <c r="K2" s="101"/>
-      <c r="L2" s="101"/>
-      <c r="M2" s="101"/>
-      <c r="N2" s="101"/>
-      <c r="O2" s="101"/>
-      <c r="P2" s="101"/>
+      <c r="A2" s="97"/>
+      <c r="B2" s="97"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="97"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="97"/>
+      <c r="I2" s="97"/>
+      <c r="J2" s="97"/>
+      <c r="K2" s="97"/>
+      <c r="L2" s="97"/>
+      <c r="M2" s="97"/>
+      <c r="N2" s="97"/>
+      <c r="O2" s="97"/>
+      <c r="P2" s="97"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A3" s="102" t="s">
+      <c r="A3" s="98" t="s">
         <v>141</v>
       </c>
-      <c r="B3" s="102"/>
-      <c r="C3" s="102"/>
-      <c r="D3" s="102"/>
-      <c r="E3" s="102"/>
-      <c r="F3" s="102"/>
-      <c r="G3" s="102"/>
-      <c r="H3" s="102"/>
-      <c r="I3" s="102"/>
-      <c r="J3" s="102"/>
-      <c r="K3" s="102"/>
-      <c r="L3" s="102"/>
-      <c r="M3" s="102"/>
-      <c r="N3" s="102"/>
-      <c r="O3" s="102"/>
-      <c r="P3" s="102"/>
+      <c r="B3" s="98"/>
+      <c r="C3" s="98"/>
+      <c r="D3" s="98"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="98"/>
+      <c r="I3" s="98"/>
+      <c r="J3" s="98"/>
+      <c r="K3" s="98"/>
+      <c r="L3" s="98"/>
+      <c r="M3" s="98"/>
+      <c r="N3" s="98"/>
+      <c r="O3" s="98"/>
+      <c r="P3" s="98"/>
     </row>
     <row r="4" spans="1:16" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">
@@ -6713,24 +6762,24 @@
       <c r="P11" s="36"/>
     </row>
     <row r="12" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="97" t="s">
+      <c r="A12" s="100" t="s">
         <v>204</v>
       </c>
-      <c r="B12" s="97"/>
-      <c r="C12" s="97"/>
-      <c r="D12" s="97"/>
-      <c r="E12" s="97"/>
-      <c r="F12" s="97"/>
-      <c r="G12" s="97"/>
-      <c r="H12" s="97"/>
-      <c r="I12" s="97"/>
-      <c r="J12" s="97"/>
-      <c r="K12" s="97"/>
-      <c r="L12" s="97"/>
-      <c r="M12" s="97"/>
-      <c r="N12" s="97"/>
-      <c r="O12" s="97"/>
-      <c r="P12" s="97"/>
+      <c r="B12" s="100"/>
+      <c r="C12" s="100"/>
+      <c r="D12" s="100"/>
+      <c r="E12" s="100"/>
+      <c r="F12" s="100"/>
+      <c r="G12" s="100"/>
+      <c r="H12" s="100"/>
+      <c r="I12" s="100"/>
+      <c r="J12" s="100"/>
+      <c r="K12" s="100"/>
+      <c r="L12" s="100"/>
+      <c r="M12" s="100"/>
+      <c r="N12" s="100"/>
+      <c r="O12" s="100"/>
+      <c r="P12" s="100"/>
     </row>
     <row r="13" spans="1:16" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="25">
@@ -6973,24 +7022,24 @@
       <c r="P17" s="36"/>
     </row>
     <row r="18" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="100" t="s">
+      <c r="A18" s="101" t="s">
         <v>244</v>
       </c>
-      <c r="B18" s="100"/>
-      <c r="C18" s="100"/>
-      <c r="D18" s="100"/>
-      <c r="E18" s="100"/>
-      <c r="F18" s="100"/>
-      <c r="G18" s="100"/>
-      <c r="H18" s="100"/>
-      <c r="I18" s="100"/>
-      <c r="J18" s="100"/>
-      <c r="K18" s="100"/>
-      <c r="L18" s="100"/>
-      <c r="M18" s="100"/>
-      <c r="N18" s="100"/>
-      <c r="O18" s="100"/>
-      <c r="P18" s="100"/>
+      <c r="B18" s="101"/>
+      <c r="C18" s="101"/>
+      <c r="D18" s="101"/>
+      <c r="E18" s="101"/>
+      <c r="F18" s="101"/>
+      <c r="G18" s="101"/>
+      <c r="H18" s="101"/>
+      <c r="I18" s="101"/>
+      <c r="J18" s="101"/>
+      <c r="K18" s="101"/>
+      <c r="L18" s="101"/>
+      <c r="M18" s="101"/>
+      <c r="N18" s="101"/>
+      <c r="O18" s="101"/>
+      <c r="P18" s="101"/>
     </row>
     <row r="19" spans="1:16" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="25">
@@ -7281,24 +7330,24 @@
       <c r="P24" s="36"/>
     </row>
     <row r="25" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="98" t="s">
+      <c r="A25" s="102" t="s">
         <v>292</v>
       </c>
-      <c r="B25" s="98"/>
-      <c r="C25" s="98"/>
-      <c r="D25" s="98"/>
-      <c r="E25" s="98"/>
-      <c r="F25" s="98"/>
-      <c r="G25" s="98"/>
-      <c r="H25" s="98"/>
-      <c r="I25" s="98"/>
-      <c r="J25" s="98"/>
-      <c r="K25" s="98"/>
-      <c r="L25" s="98"/>
-      <c r="M25" s="98"/>
-      <c r="N25" s="98"/>
-      <c r="O25" s="98"/>
-      <c r="P25" s="98"/>
+      <c r="B25" s="102"/>
+      <c r="C25" s="102"/>
+      <c r="D25" s="102"/>
+      <c r="E25" s="102"/>
+      <c r="F25" s="102"/>
+      <c r="G25" s="102"/>
+      <c r="H25" s="102"/>
+      <c r="I25" s="102"/>
+      <c r="J25" s="102"/>
+      <c r="K25" s="102"/>
+      <c r="L25" s="102"/>
+      <c r="M25" s="102"/>
+      <c r="N25" s="102"/>
+      <c r="O25" s="102"/>
+      <c r="P25" s="102"/>
     </row>
     <row r="26" spans="1:16" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="25">
@@ -7801,24 +7850,24 @@
       <c r="P36" s="36"/>
     </row>
     <row r="37" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="98" t="s">
+      <c r="A37" s="102" t="s">
         <v>370</v>
       </c>
-      <c r="B37" s="98"/>
-      <c r="C37" s="98"/>
-      <c r="D37" s="98"/>
-      <c r="E37" s="98"/>
-      <c r="F37" s="98"/>
-      <c r="G37" s="98"/>
-      <c r="H37" s="98"/>
-      <c r="I37" s="98"/>
-      <c r="J37" s="98"/>
-      <c r="K37" s="98"/>
-      <c r="L37" s="98"/>
-      <c r="M37" s="98"/>
-      <c r="N37" s="98"/>
-      <c r="O37" s="98"/>
-      <c r="P37" s="98"/>
+      <c r="B37" s="102"/>
+      <c r="C37" s="102"/>
+      <c r="D37" s="102"/>
+      <c r="E37" s="102"/>
+      <c r="F37" s="102"/>
+      <c r="G37" s="102"/>
+      <c r="H37" s="102"/>
+      <c r="I37" s="102"/>
+      <c r="J37" s="102"/>
+      <c r="K37" s="102"/>
+      <c r="L37" s="102"/>
+      <c r="M37" s="102"/>
+      <c r="N37" s="102"/>
+      <c r="O37" s="102"/>
+      <c r="P37" s="102"/>
     </row>
     <row r="38" spans="1:16" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="25">
@@ -8013,24 +8062,24 @@
       <c r="P41" s="36"/>
     </row>
     <row r="42" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="100" t="s">
+      <c r="A42" s="101" t="s">
         <v>399</v>
       </c>
-      <c r="B42" s="100"/>
-      <c r="C42" s="100"/>
-      <c r="D42" s="100"/>
-      <c r="E42" s="100"/>
-      <c r="F42" s="100"/>
-      <c r="G42" s="100"/>
-      <c r="H42" s="100"/>
-      <c r="I42" s="100"/>
-      <c r="J42" s="100"/>
-      <c r="K42" s="100"/>
-      <c r="L42" s="100"/>
-      <c r="M42" s="100"/>
-      <c r="N42" s="100"/>
-      <c r="O42" s="100"/>
-      <c r="P42" s="100"/>
+      <c r="B42" s="101"/>
+      <c r="C42" s="101"/>
+      <c r="D42" s="101"/>
+      <c r="E42" s="101"/>
+      <c r="F42" s="101"/>
+      <c r="G42" s="101"/>
+      <c r="H42" s="101"/>
+      <c r="I42" s="101"/>
+      <c r="J42" s="101"/>
+      <c r="K42" s="101"/>
+      <c r="L42" s="101"/>
+      <c r="M42" s="101"/>
+      <c r="N42" s="101"/>
+      <c r="O42" s="101"/>
+      <c r="P42" s="101"/>
     </row>
     <row r="43" spans="1:16" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="25">
@@ -8321,24 +8370,24 @@
       <c r="P48" s="36"/>
     </row>
     <row r="49" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="98" t="s">
+      <c r="A49" s="102" t="s">
         <v>443</v>
       </c>
-      <c r="B49" s="98"/>
-      <c r="C49" s="98"/>
-      <c r="D49" s="98"/>
-      <c r="E49" s="98"/>
-      <c r="F49" s="98"/>
-      <c r="G49" s="98"/>
-      <c r="H49" s="98"/>
-      <c r="I49" s="98"/>
-      <c r="J49" s="98"/>
-      <c r="K49" s="98"/>
-      <c r="L49" s="98"/>
-      <c r="M49" s="98"/>
-      <c r="N49" s="98"/>
-      <c r="O49" s="98"/>
-      <c r="P49" s="98"/>
+      <c r="B49" s="102"/>
+      <c r="C49" s="102"/>
+      <c r="D49" s="102"/>
+      <c r="E49" s="102"/>
+      <c r="F49" s="102"/>
+      <c r="G49" s="102"/>
+      <c r="H49" s="102"/>
+      <c r="I49" s="102"/>
+      <c r="J49" s="102"/>
+      <c r="K49" s="102"/>
+      <c r="L49" s="102"/>
+      <c r="M49" s="102"/>
+      <c r="N49" s="102"/>
+      <c r="O49" s="102"/>
+      <c r="P49" s="102"/>
     </row>
     <row r="50" spans="1:16" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="25">
@@ -8533,24 +8582,24 @@
       <c r="P53" s="36"/>
     </row>
     <row r="54" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="97" t="s">
+      <c r="A54" s="100" t="s">
         <v>471</v>
       </c>
-      <c r="B54" s="97"/>
-      <c r="C54" s="97"/>
-      <c r="D54" s="97"/>
-      <c r="E54" s="97"/>
-      <c r="F54" s="97"/>
-      <c r="G54" s="97"/>
-      <c r="H54" s="97"/>
-      <c r="I54" s="97"/>
-      <c r="J54" s="97"/>
-      <c r="K54" s="97"/>
-      <c r="L54" s="97"/>
-      <c r="M54" s="97"/>
-      <c r="N54" s="97"/>
-      <c r="O54" s="97"/>
-      <c r="P54" s="97"/>
+      <c r="B54" s="100"/>
+      <c r="C54" s="100"/>
+      <c r="D54" s="100"/>
+      <c r="E54" s="100"/>
+      <c r="F54" s="100"/>
+      <c r="G54" s="100"/>
+      <c r="H54" s="100"/>
+      <c r="I54" s="100"/>
+      <c r="J54" s="100"/>
+      <c r="K54" s="100"/>
+      <c r="L54" s="100"/>
+      <c r="M54" s="100"/>
+      <c r="N54" s="100"/>
+      <c r="O54" s="100"/>
+      <c r="P54" s="100"/>
     </row>
     <row r="55" spans="1:16" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="25">
@@ -8793,24 +8842,24 @@
       <c r="P59" s="36"/>
     </row>
     <row r="60" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="98" t="s">
+      <c r="A60" s="102" t="s">
         <v>508</v>
       </c>
-      <c r="B60" s="98"/>
-      <c r="C60" s="98"/>
-      <c r="D60" s="98"/>
-      <c r="E60" s="98"/>
-      <c r="F60" s="98"/>
-      <c r="G60" s="98"/>
-      <c r="H60" s="98"/>
-      <c r="I60" s="98"/>
-      <c r="J60" s="98"/>
-      <c r="K60" s="98"/>
-      <c r="L60" s="98"/>
-      <c r="M60" s="98"/>
-      <c r="N60" s="98"/>
-      <c r="O60" s="98"/>
-      <c r="P60" s="98"/>
+      <c r="B60" s="102"/>
+      <c r="C60" s="102"/>
+      <c r="D60" s="102"/>
+      <c r="E60" s="102"/>
+      <c r="F60" s="102"/>
+      <c r="G60" s="102"/>
+      <c r="H60" s="102"/>
+      <c r="I60" s="102"/>
+      <c r="J60" s="102"/>
+      <c r="K60" s="102"/>
+      <c r="L60" s="102"/>
+      <c r="M60" s="102"/>
+      <c r="N60" s="102"/>
+      <c r="O60" s="102"/>
+      <c r="P60" s="102"/>
     </row>
     <row r="61" spans="1:16" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="25">
@@ -9005,24 +9054,24 @@
       <c r="P64" s="36"/>
     </row>
     <row r="65" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="98" t="s">
+      <c r="A65" s="102" t="s">
         <v>537</v>
       </c>
-      <c r="B65" s="98"/>
-      <c r="C65" s="98"/>
-      <c r="D65" s="98"/>
-      <c r="E65" s="98"/>
-      <c r="F65" s="98"/>
-      <c r="G65" s="98"/>
-      <c r="H65" s="98"/>
-      <c r="I65" s="98"/>
-      <c r="J65" s="98"/>
-      <c r="K65" s="98"/>
-      <c r="L65" s="98"/>
-      <c r="M65" s="98"/>
-      <c r="N65" s="98"/>
-      <c r="O65" s="98"/>
-      <c r="P65" s="98"/>
+      <c r="B65" s="102"/>
+      <c r="C65" s="102"/>
+      <c r="D65" s="102"/>
+      <c r="E65" s="102"/>
+      <c r="F65" s="102"/>
+      <c r="G65" s="102"/>
+      <c r="H65" s="102"/>
+      <c r="I65" s="102"/>
+      <c r="J65" s="102"/>
+      <c r="K65" s="102"/>
+      <c r="L65" s="102"/>
+      <c r="M65" s="102"/>
+      <c r="N65" s="102"/>
+      <c r="O65" s="102"/>
+      <c r="P65" s="102"/>
     </row>
     <row r="66" spans="1:16" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="25">
@@ -9218,11 +9267,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A1:P2"/>
-    <mergeCell ref="A3:P3"/>
-    <mergeCell ref="A5:P5"/>
-    <mergeCell ref="A12:P12"/>
-    <mergeCell ref="A18:P18"/>
     <mergeCell ref="A54:P54"/>
     <mergeCell ref="A60:P60"/>
     <mergeCell ref="A65:P65"/>
@@ -9231,6 +9275,11 @@
     <mergeCell ref="A37:P37"/>
     <mergeCell ref="A42:P42"/>
     <mergeCell ref="A49:P49"/>
+    <mergeCell ref="A1:P2"/>
+    <mergeCell ref="A3:P3"/>
+    <mergeCell ref="A5:P5"/>
+    <mergeCell ref="A12:P12"/>
+    <mergeCell ref="A18:P18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -9260,53 +9309,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="97" t="s">
         <v>567</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="101"/>
-      <c r="I1" s="101"/>
-      <c r="J1" s="101"/>
-      <c r="K1" s="101"/>
-      <c r="L1" s="101"/>
-      <c r="M1" s="101"/>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" s="101"/>
-      <c r="B2" s="101"/>
-      <c r="C2" s="101"/>
-      <c r="D2" s="101"/>
-      <c r="E2" s="101"/>
-      <c r="F2" s="101"/>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="101"/>
-      <c r="J2" s="101"/>
-      <c r="K2" s="101"/>
-      <c r="L2" s="101"/>
-      <c r="M2" s="101"/>
+      <c r="A2" s="97"/>
+      <c r="B2" s="97"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="97"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="97"/>
+      <c r="I2" s="97"/>
+      <c r="J2" s="97"/>
+      <c r="K2" s="97"/>
+      <c r="L2" s="97"/>
+      <c r="M2" s="97"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3" s="102" t="s">
+      <c r="A3" s="98" t="s">
         <v>568</v>
       </c>
-      <c r="B3" s="102"/>
-      <c r="C3" s="102"/>
-      <c r="D3" s="102"/>
-      <c r="E3" s="102"/>
-      <c r="F3" s="102"/>
-      <c r="G3" s="102"/>
-      <c r="H3" s="102"/>
-      <c r="I3" s="102"/>
-      <c r="J3" s="102"/>
-      <c r="K3" s="102"/>
-      <c r="L3" s="102"/>
-      <c r="M3" s="102"/>
+      <c r="B3" s="98"/>
+      <c r="C3" s="98"/>
+      <c r="D3" s="98"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="98"/>
+      <c r="I3" s="98"/>
+      <c r="J3" s="98"/>
+      <c r="K3" s="98"/>
+      <c r="L3" s="98"/>
+      <c r="M3" s="98"/>
     </row>
     <row r="4" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">
@@ -10221,56 +10270,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="97" t="s">
         <v>703</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="101"/>
-      <c r="I1" s="101"/>
-      <c r="J1" s="101"/>
-      <c r="K1" s="101"/>
-      <c r="L1" s="101"/>
-      <c r="M1" s="101"/>
-      <c r="N1" s="101"/>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" s="101"/>
-      <c r="B2" s="101"/>
-      <c r="C2" s="101"/>
-      <c r="D2" s="101"/>
-      <c r="E2" s="101"/>
-      <c r="F2" s="101"/>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="101"/>
-      <c r="J2" s="101"/>
-      <c r="K2" s="101"/>
-      <c r="L2" s="101"/>
-      <c r="M2" s="101"/>
-      <c r="N2" s="101"/>
+      <c r="A2" s="97"/>
+      <c r="B2" s="97"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="97"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="97"/>
+      <c r="I2" s="97"/>
+      <c r="J2" s="97"/>
+      <c r="K2" s="97"/>
+      <c r="L2" s="97"/>
+      <c r="M2" s="97"/>
+      <c r="N2" s="97"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A3" s="102" t="s">
+      <c r="A3" s="98" t="s">
         <v>704</v>
       </c>
-      <c r="B3" s="102"/>
-      <c r="C3" s="102"/>
-      <c r="D3" s="102"/>
-      <c r="E3" s="102"/>
-      <c r="F3" s="102"/>
-      <c r="G3" s="102"/>
-      <c r="H3" s="102"/>
-      <c r="I3" s="102"/>
-      <c r="J3" s="102"/>
-      <c r="K3" s="102"/>
-      <c r="L3" s="102"/>
-      <c r="M3" s="102"/>
-      <c r="N3" s="102"/>
+      <c r="B3" s="98"/>
+      <c r="C3" s="98"/>
+      <c r="D3" s="98"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="98"/>
+      <c r="I3" s="98"/>
+      <c r="J3" s="98"/>
+      <c r="K3" s="98"/>
+      <c r="L3" s="98"/>
+      <c r="M3" s="98"/>
+      <c r="N3" s="98"/>
     </row>
     <row r="4" spans="1:14" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">
@@ -11140,7 +11189,7 @@
   <sheetPr>
     <tabColor rgb="FF1D4ED8"/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -11154,44 +11203,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="97" t="s">
         <v>831</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="101"/>
-      <c r="I1" s="101"/>
-      <c r="J1" s="101"/>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="101"/>
-      <c r="B2" s="101"/>
-      <c r="C2" s="101"/>
-      <c r="D2" s="101"/>
-      <c r="E2" s="101"/>
-      <c r="F2" s="101"/>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="101"/>
-      <c r="J2" s="101"/>
+      <c r="A2" s="97"/>
+      <c r="B2" s="97"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="97"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="97"/>
+      <c r="I2" s="97"/>
+      <c r="J2" s="97"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="102" t="s">
+      <c r="A3" s="98" t="s">
         <v>832</v>
       </c>
-      <c r="B3" s="102"/>
-      <c r="C3" s="102"/>
-      <c r="D3" s="102"/>
-      <c r="E3" s="102"/>
-      <c r="F3" s="102"/>
-      <c r="G3" s="102"/>
-      <c r="H3" s="102"/>
-      <c r="I3" s="102"/>
-      <c r="J3" s="102"/>
+      <c r="B3" s="98"/>
+      <c r="C3" s="98"/>
+      <c r="D3" s="98"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="98"/>
+      <c r="I3" s="98"/>
+      <c r="J3" s="98"/>
     </row>
     <row r="4" spans="1:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">
@@ -11927,6 +11976,233 @@
       </c>
       <c r="J26" s="82" t="s">
         <v>841</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A27" s="113">
+        <v>23</v>
+      </c>
+      <c r="B27" s="114">
+        <v>46268</v>
+      </c>
+      <c r="C27" t="s">
+        <v>1028</v>
+      </c>
+      <c r="D27" t="s">
+        <v>99</v>
+      </c>
+      <c r="E27" t="s">
+        <v>100</v>
+      </c>
+      <c r="F27" t="s">
+        <v>101</v>
+      </c>
+      <c r="G27" t="s">
+        <v>103</v>
+      </c>
+      <c r="H27">
+        <v>4.2</v>
+      </c>
+      <c r="I27" t="s">
+        <v>1029</v>
+      </c>
+      <c r="J27" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A28" s="113">
+        <v>24</v>
+      </c>
+      <c r="B28" s="114">
+        <v>46273</v>
+      </c>
+      <c r="C28" t="s">
+        <v>1030</v>
+      </c>
+      <c r="D28" t="s">
+        <v>106</v>
+      </c>
+      <c r="E28" t="s">
+        <v>107</v>
+      </c>
+      <c r="F28" t="s">
+        <v>108</v>
+      </c>
+      <c r="G28" t="s">
+        <v>110</v>
+      </c>
+      <c r="H28">
+        <v>2.4</v>
+      </c>
+      <c r="I28" t="s">
+        <v>1031</v>
+      </c>
+      <c r="J28" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A29" s="113">
+        <v>25</v>
+      </c>
+      <c r="B29" s="114">
+        <v>46275</v>
+      </c>
+      <c r="C29" t="s">
+        <v>1028</v>
+      </c>
+      <c r="D29" t="s">
+        <v>116</v>
+      </c>
+      <c r="E29" t="s">
+        <v>117</v>
+      </c>
+      <c r="F29" t="s">
+        <v>108</v>
+      </c>
+      <c r="G29" t="s">
+        <v>110</v>
+      </c>
+      <c r="H29">
+        <v>2.1</v>
+      </c>
+      <c r="I29" t="s">
+        <v>1032</v>
+      </c>
+      <c r="J29" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A30" s="113">
+        <v>2</v>
+      </c>
+      <c r="B30" s="114">
+        <v>46280</v>
+      </c>
+      <c r="C30" t="s">
+        <v>1030</v>
+      </c>
+      <c r="D30" t="s">
+        <v>120</v>
+      </c>
+      <c r="E30" t="s">
+        <v>121</v>
+      </c>
+      <c r="F30" t="s">
+        <v>101</v>
+      </c>
+      <c r="G30" t="s">
+        <v>103</v>
+      </c>
+      <c r="H30">
+        <v>3.5</v>
+      </c>
+      <c r="I30" t="s">
+        <v>1033</v>
+      </c>
+      <c r="J30" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A31" s="113">
+        <v>627</v>
+      </c>
+      <c r="B31" s="114">
+        <v>46282</v>
+      </c>
+      <c r="C31" t="s">
+        <v>1028</v>
+      </c>
+      <c r="D31" t="s">
+        <v>124</v>
+      </c>
+      <c r="E31" t="s">
+        <v>125</v>
+      </c>
+      <c r="F31" t="s">
+        <v>108</v>
+      </c>
+      <c r="G31" t="s">
+        <v>110</v>
+      </c>
+      <c r="H31">
+        <v>1.8</v>
+      </c>
+      <c r="I31" t="s">
+        <v>1034</v>
+      </c>
+      <c r="J31" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A32" s="113">
+        <v>28</v>
+      </c>
+      <c r="B32" s="114">
+        <v>46287</v>
+      </c>
+      <c r="C32" t="s">
+        <v>1030</v>
+      </c>
+      <c r="D32" t="s">
+        <v>131</v>
+      </c>
+      <c r="E32" t="s">
+        <v>132</v>
+      </c>
+      <c r="F32" t="s">
+        <v>108</v>
+      </c>
+      <c r="G32" t="s">
+        <v>110</v>
+      </c>
+      <c r="H32">
+        <v>1.5</v>
+      </c>
+      <c r="I32" t="s">
+        <v>1035</v>
+      </c>
+      <c r="J32" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A33" s="113"/>
+      <c r="B33" s="114">
+        <v>46289</v>
+      </c>
+      <c r="C33" t="s">
+        <v>1028</v>
+      </c>
+      <c r="D33" t="s">
+        <v>134</v>
+      </c>
+      <c r="E33" t="s">
+        <v>135</v>
+      </c>
+      <c r="F33" t="s">
+        <v>108</v>
+      </c>
+      <c r="G33" t="s">
+        <v>110</v>
+      </c>
+      <c r="H33">
+        <v>1.5</v>
+      </c>
+      <c r="I33" t="s">
+        <v>1036</v>
+      </c>
+      <c r="J33" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A34" s="113">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -11960,44 +12236,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="97" t="s">
         <v>854</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="101"/>
-      <c r="I1" s="101"/>
-      <c r="J1" s="101"/>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="101"/>
-      <c r="B2" s="101"/>
-      <c r="C2" s="101"/>
-      <c r="D2" s="101"/>
-      <c r="E2" s="101"/>
-      <c r="F2" s="101"/>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="101"/>
-      <c r="J2" s="101"/>
+      <c r="A2" s="97"/>
+      <c r="B2" s="97"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="97"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="97"/>
+      <c r="I2" s="97"/>
+      <c r="J2" s="97"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="102" t="s">
+      <c r="A3" s="98" t="s">
         <v>855</v>
       </c>
-      <c r="B3" s="102"/>
-      <c r="C3" s="102"/>
-      <c r="D3" s="102"/>
-      <c r="E3" s="102"/>
-      <c r="F3" s="102"/>
-      <c r="G3" s="102"/>
-      <c r="H3" s="102"/>
-      <c r="I3" s="102"/>
-      <c r="J3" s="102"/>
+      <c r="B3" s="98"/>
+      <c r="C3" s="98"/>
+      <c r="D3" s="98"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="98"/>
+      <c r="I3" s="98"/>
+      <c r="J3" s="98"/>
     </row>
     <row r="4" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">
@@ -12319,56 +12595,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="97" t="s">
         <v>915</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="101"/>
-      <c r="I1" s="101"/>
-      <c r="J1" s="101"/>
-      <c r="K1" s="101"/>
-      <c r="L1" s="101"/>
-      <c r="M1" s="101"/>
-      <c r="N1" s="101"/>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" s="101"/>
-      <c r="B2" s="101"/>
-      <c r="C2" s="101"/>
-      <c r="D2" s="101"/>
-      <c r="E2" s="101"/>
-      <c r="F2" s="101"/>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="101"/>
-      <c r="J2" s="101"/>
-      <c r="K2" s="101"/>
-      <c r="L2" s="101"/>
-      <c r="M2" s="101"/>
-      <c r="N2" s="101"/>
+      <c r="A2" s="97"/>
+      <c r="B2" s="97"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="97"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="97"/>
+      <c r="I2" s="97"/>
+      <c r="J2" s="97"/>
+      <c r="K2" s="97"/>
+      <c r="L2" s="97"/>
+      <c r="M2" s="97"/>
+      <c r="N2" s="97"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A3" s="102" t="s">
+      <c r="A3" s="98" t="s">
         <v>916</v>
       </c>
-      <c r="B3" s="102"/>
-      <c r="C3" s="102"/>
-      <c r="D3" s="102"/>
-      <c r="E3" s="102"/>
-      <c r="F3" s="102"/>
-      <c r="G3" s="102"/>
-      <c r="H3" s="102"/>
-      <c r="I3" s="102"/>
-      <c r="J3" s="102"/>
-      <c r="K3" s="102"/>
-      <c r="L3" s="102"/>
-      <c r="M3" s="102"/>
-      <c r="N3" s="102"/>
+      <c r="B3" s="98"/>
+      <c r="C3" s="98"/>
+      <c r="D3" s="98"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="98"/>
+      <c r="I3" s="98"/>
+      <c r="J3" s="98"/>
+      <c r="K3" s="98"/>
+      <c r="L3" s="98"/>
+      <c r="M3" s="98"/>
+      <c r="N3" s="98"/>
     </row>
     <row r="4" spans="1:14" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">
@@ -12741,44 +13017,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="97" t="s">
         <v>951</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="101"/>
-      <c r="I1" s="101"/>
-      <c r="J1" s="101"/>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="101"/>
-      <c r="B2" s="101"/>
-      <c r="C2" s="101"/>
-      <c r="D2" s="101"/>
-      <c r="E2" s="101"/>
-      <c r="F2" s="101"/>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="101"/>
-      <c r="J2" s="101"/>
+      <c r="A2" s="97"/>
+      <c r="B2" s="97"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="97"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="97"/>
+      <c r="I2" s="97"/>
+      <c r="J2" s="97"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="102" t="s">
+      <c r="A3" s="98" t="s">
         <v>952</v>
       </c>
-      <c r="B3" s="102"/>
-      <c r="C3" s="102"/>
-      <c r="D3" s="102"/>
-      <c r="E3" s="102"/>
-      <c r="F3" s="102"/>
-      <c r="G3" s="102"/>
-      <c r="H3" s="102"/>
-      <c r="I3" s="102"/>
-      <c r="J3" s="102"/>
+      <c r="B3" s="98"/>
+      <c r="C3" s="98"/>
+      <c r="D3" s="98"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="98"/>
+      <c r="I3" s="98"/>
+      <c r="J3" s="98"/>
     </row>
     <row r="4" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">

</xml_diff>